<commit_message>
fix(jintan-weekly-report): align config, docs, engine and validators
- Update DEPLOYMENT.md to reflect existing v9 engine and validators
- Make generate-milestone-image.py read config.yaml instead of hardcoding
- Bump milestone image font sizes to >=28px in config.yaml
- Fix report_engine_v9.py console print keys and duplicate heading
- Unify clean_notes week range to Mon-Sun
- Show progress% in next_week plans and sanitize 进展中
- Fix eastAsia font for 暂无 placeholders
- Update validate_report_tone risk regex and quantification rules
- Simplify empty-task placeholder check in validate_weekly_report
- Refresh data and regenerate weekly report; both QA checks PASS

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jintan-weekly-report-sop/data/金坛二期项目跟进表.xlsx
+++ b/jintan-weekly-report-sop/data/金坛二期项目跟进表.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="276">
   <si>
     <t>序号</t>
   </si>
@@ -166,9 +166,6 @@
   </si>
   <si>
     <t>6月5日</t>
-  </si>
-  <si>
-    <t>95%</t>
   </si>
   <si>
     <t>0611：李江跟分院签字预计在6月15-6月18号完成
@@ -199,7 +196,17 @@
     <t>高保真设计</t>
   </si>
   <si>
-    <t>1、已与薛埠分院调研，分院提出3点修改要求
+    <t>6月26日</t>
+  </si>
+  <si>
+    <t>99%</t>
+  </si>
+  <si>
+    <t>6月29日</t>
+  </si>
+  <si>
+    <t>0626:已经根据分院反馈意见和总院沟通，完善最终的指标清单
+1、已与薛埠分院调研，分院提出3点修改要求
 2、已与公卫进行沟通确认</t>
   </si>
   <si>
@@ -215,9 +222,6 @@
     <t>90%</t>
   </si>
   <si>
-    <t>未开始</t>
-  </si>
-  <si>
     <t>需要确认评审的形式及要求</t>
   </si>
   <si>
@@ -233,19 +237,17 @@
     <t>王雪娇</t>
   </si>
   <si>
-    <t>6月8日</t>
-  </si>
-  <si>
-    <t>6月30日</t>
+    <t>6月12日</t>
+  </si>
+  <si>
+    <t>7月12日</t>
   </si>
   <si>
     <t>1%</t>
   </si>
   <si>
-    <t>6月12日</t>
-  </si>
-  <si>
-    <t>0611 李江已和卫宁方一期推进</t>
+    <t>0626 已经签订合同，需要移动打款后推进
+0611 李江已和卫宁方一期推进</t>
   </si>
   <si>
     <t>数据应用开发</t>
@@ -260,16 +262,17 @@
     <t>6月10日</t>
   </si>
   <si>
-    <t>6月18日</t>
-  </si>
-  <si>
-    <t>8%</t>
+    <t>7月3日</t>
+  </si>
+  <si>
+    <t>30%</t>
   </si>
   <si>
     <t>6月4日</t>
   </si>
   <si>
-    <t>0611：卫宁数据开发进行中，需要提供数据字典给smartbi
+    <t>0626：smartbi已经利用测试数据开发了页面，目前稳序进展中
+0611：卫宁数据开发进行中，需要提供数据字典给smartbi
 0609：已发送开发所需账号密码，已提供原型图的源文件切图
 0604:可以开始推进，发送原型材料，通知smart可以安排资源进场</t>
   </si>
@@ -283,10 +286,10 @@
     <t>《0601.自测报告》</t>
   </si>
   <si>
-    <t>6月20日</t>
-  </si>
-  <si>
-    <t>7月3日</t>
+    <t>7月6日</t>
+  </si>
+  <si>
+    <t>未开始</t>
   </si>
   <si>
     <t>UAT测试及系统缺陷修复</t>
@@ -322,10 +325,8 @@
     <t>5月20日</t>
   </si>
   <si>
-    <t>70%</t>
-  </si>
-  <si>
-    <t>0605：消化内科反馈原型图暂无问题
+    <t>0618：周科反馈大内科暂无问题，下周再跟周科一起去其他科室调研
+0605：消化内科反馈原型图暂无问题
 0529:已与消化内科进行调研，后续调整原型
 0527内部再出一版，再找消化内科调研下
 0428:针对消化内科、心内科梳理仿真数据供调研使用</t>
@@ -334,9 +335,6 @@
     <t>陆婷婷、李新元</t>
   </si>
   <si>
-    <t>60%</t>
-  </si>
-  <si>
     <t>0605：消化内科反馈初版暂无问题
 0603：和消化内科确认原型</t>
   </si>
@@ -350,7 +348,8 @@
     <t>5月18日</t>
   </si>
   <si>
-    <t>0605：消化内科反馈初版暂无问题，需要进一步美化UI
+    <t>0618：周科反馈跟其他几个科室调研过，暂无修改修改的问题，下周再找几个科室进行调研
+0605：消化内科反馈初版暂无问题，需要进一步美化UI
 0603：和消化内科确认原型
 0515：21号出一版，内部讨论</t>
   </si>
@@ -361,51 +360,70 @@
     <t>原型图外部评审</t>
   </si>
   <si>
+    <t>6月8日</t>
+  </si>
+  <si>
+    <t>95%</t>
+  </si>
+  <si>
+    <t>0626 根据调研的建议再修改一下原型图，下周上半周再补一个大内科的签字
+0618：美化UI中，预计下周跟周科一起科室调研
+0612：美化UI后发给李江了，请他发给周科</t>
+  </si>
+  <si>
+    <t>数据开发</t>
+  </si>
+  <si>
+    <t>7月24日</t>
+  </si>
+  <si>
+    <t>0622：已跟火树反馈需要取数</t>
+  </si>
+  <si>
+    <t>分析看板多维度联动、下钻功能开发</t>
+  </si>
+  <si>
+    <t>7月17日</t>
+  </si>
+  <si>
+    <t>0629号可通知smart开发</t>
+  </si>
+  <si>
+    <t>7月25日</t>
+  </si>
+  <si>
+    <t>8月10日</t>
+  </si>
+  <si>
+    <t>8月15日</t>
+  </si>
+  <si>
+    <t>（调研科室签字）</t>
+  </si>
+  <si>
+    <t>8月5日</t>
+  </si>
+  <si>
+    <t>8月25日</t>
+  </si>
+  <si>
+    <t>"掌上院情" 移动决策</t>
+  </si>
+  <si>
+    <t>《0303.场景原型图》内部初稿</t>
+  </si>
+  <si>
+    <t>5月10日</t>
+  </si>
+  <si>
     <t>80%</t>
-  </si>
-  <si>
-    <t>0618：美化UI中，预计下周跟周科一起科室调研
-0612：美化UI后发给李江了，请他发给周科</t>
-  </si>
-  <si>
-    <t>数据开发</t>
-  </si>
-  <si>
-    <t>6月22日</t>
-  </si>
-  <si>
-    <t>7月10日</t>
-  </si>
-  <si>
-    <t>分析看板多维度联动、下钻功能开发</t>
-  </si>
-  <si>
-    <t>8月20日</t>
-  </si>
-  <si>
-    <t>7月15日</t>
-  </si>
-  <si>
-    <t>8月5日</t>
-  </si>
-  <si>
-    <t>"掌上院情" 移动决策</t>
-  </si>
-  <si>
-    <t>《0303.场景原型图》内部初稿</t>
-  </si>
-  <si>
-    <t>5月10日</t>
   </si>
   <si>
     <t>0612 已完成初稿，下周需要优化原型和高保真设计
 0605 设计一版原型图初稿，用于内部讨论内部讨论</t>
   </si>
   <si>
-    <t>6月15日</t>
-  </si>
-  <si>
-    <t>6月26日</t>
+    <t>6月30日</t>
   </si>
   <si>
     <t>https://modao.cc/proto/tOvCz41NtfbmtugyXxVnGo/sharing?view_mode=read_only&amp;screen=rbpVK8XTcI6hcrnIe #掌上院情-分享</t>
@@ -414,13 +432,7 @@
     <t>6月28日</t>
   </si>
   <si>
-    <t>7月17日</t>
-  </si>
-  <si>
     <t>移动端H5页面适配与图表渲染开发</t>
-  </si>
-  <si>
-    <t>8月15日</t>
   </si>
   <si>
     <t>8月28日</t>
@@ -589,9 +601,6 @@
   </si>
   <si>
     <t>已完成</t>
-  </si>
-  <si>
-    <t>30%</t>
   </si>
   <si>
     <t>项目上线</t>
@@ -639,6 +648,9 @@
 《1001.试运行报告》
 《1002.平台监控报告》
 《1101.项目验收书》</t>
+  </si>
+  <si>
+    <t>60%</t>
   </si>
   <si>
     <t>免费维保1年</t>
@@ -1495,30 +1507,30 @@
         <v>48</v>
       </c>
       <c r="J7" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="K7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L7" t="s">
         <v>39</v>
       </c>
       <c r="N7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>52</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>53</v>
-      </c>
-      <c r="F8" t="s">
-        <v>54</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
@@ -1544,13 +1556,13 @@
     </row>
     <row r="9" spans="1:14">
       <c r="D9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" t="s">
         <v>53</v>
-      </c>
-      <c r="F9" t="s">
-        <v>54</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
@@ -1559,27 +1571,27 @@
         <v>47</v>
       </c>
       <c r="I9" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="J9" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="K9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="L9" t="s">
         <v>39</v>
       </c>
       <c r="M9" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="N9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="D10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
@@ -1591,51 +1603,51 @@
         <v>18</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="J10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K10" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="N10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="C11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
         <v>18</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K11" t="s">
         <v>21</v>
       </c>
       <c r="L11" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="N11" t="s">
         <v>71</v>
@@ -1652,7 +1664,7 @@
         <v>74</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G12" t="s">
         <v>18</v>
@@ -1687,7 +1699,7 @@
         <v>82</v>
       </c>
       <c r="F13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G13" t="s">
         <v>18</v>
@@ -1696,10 +1708,10 @@
         <v>83</v>
       </c>
       <c r="I13" t="s">
+        <v>76</v>
+      </c>
+      <c r="K13" t="s">
         <v>84</v>
-      </c>
-      <c r="K13" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1707,7 +1719,7 @@
         <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G14" t="s">
         <v>18</v>
@@ -1719,7 +1731,7 @@
         <v>87</v>
       </c>
       <c r="K14" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -1730,7 +1742,7 @@
         <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
         <v>18</v>
@@ -1742,7 +1754,7 @@
         <v>91</v>
       </c>
       <c r="K15" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -1774,13 +1786,13 @@
         <v>95</v>
       </c>
       <c r="J16" t="s">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="K16" t="s">
         <v>21</v>
       </c>
       <c r="N16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -1791,7 +1803,7 @@
         <v>45</v>
       </c>
       <c r="F17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G17" t="s">
         <v>18</v>
@@ -1800,112 +1812,115 @@
         <v>47</v>
       </c>
       <c r="I17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="J17" t="s">
-        <v>99</v>
+        <v>24</v>
       </c>
       <c r="K17" t="s">
         <v>21</v>
       </c>
       <c r="N17" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="C18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F18" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" t="s">
         <v>101</v>
       </c>
-      <c r="E18" t="s">
-        <v>53</v>
-      </c>
-      <c r="F18" t="s">
-        <v>102</v>
-      </c>
-      <c r="G18" t="s">
-        <v>18</v>
-      </c>
-      <c r="H18" t="s">
-        <v>103</v>
-      </c>
       <c r="I18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J18" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="K18" t="s">
         <v>21</v>
       </c>
       <c r="L18" t="s">
+        <v>101</v>
+      </c>
+      <c r="N18" t="s">
+        <v>102</v>
+      </c>
+      <c r="O18" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="N18" t="s">
-        <v>104</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="D19" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E19" t="s">
         <v>37</v>
       </c>
       <c r="F19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G19" t="s">
         <v>18</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="I19" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="J19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K19" t="s">
         <v>21</v>
       </c>
       <c r="L19" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="N19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="C20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" t="s">
+        <v>100</v>
+      </c>
+      <c r="G20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" t="s">
+        <v>83</v>
+      </c>
+      <c r="I20" t="s">
         <v>109</v>
       </c>
-      <c r="D20" t="s">
-        <v>64</v>
-      </c>
-      <c r="E20" t="s">
-        <v>65</v>
-      </c>
-      <c r="F20" t="s">
-        <v>102</v>
-      </c>
-      <c r="G20" t="s">
-        <v>18</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="K20" t="s">
+        <v>84</v>
+      </c>
+      <c r="N20" t="s">
         <v>110</v>
-      </c>
-      <c r="I20" t="s">
-        <v>111</v>
-      </c>
-      <c r="K20" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -1913,25 +1928,28 @@
         <v>72</v>
       </c>
       <c r="D21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E21" t="s">
         <v>74</v>
       </c>
       <c r="F21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G21" t="s">
         <v>18</v>
       </c>
       <c r="H21" t="s">
-        <v>110</v>
+        <v>57</v>
       </c>
       <c r="I21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K21" t="s">
-        <v>61</v>
+        <v>21</v>
+      </c>
+      <c r="N21" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -1945,19 +1963,19 @@
         <v>82</v>
       </c>
       <c r="F22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G22" t="s">
         <v>18</v>
       </c>
       <c r="H22" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K22" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -1965,7 +1983,7 @@
         <v>85</v>
       </c>
       <c r="F23" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G23" t="s">
         <v>18</v>
@@ -1974,10 +1992,13 @@
         <v>114</v>
       </c>
       <c r="I23" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="K23" t="s">
-        <v>61</v>
+        <v>84</v>
+      </c>
+      <c r="N23" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -1988,19 +2009,19 @@
         <v>89</v>
       </c>
       <c r="F24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G24" t="s">
         <v>18</v>
       </c>
       <c r="H24" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I24" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="K24" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -2008,89 +2029,89 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G25" t="s">
         <v>18</v>
       </c>
       <c r="H25" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I25" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="J25" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="K25" t="s">
         <v>21</v>
       </c>
       <c r="N25" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="D26" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E26" t="s">
         <v>37</v>
       </c>
       <c r="F26" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G26" t="s">
         <v>18</v>
       </c>
       <c r="H26" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="I26" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="K26" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="C27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F27" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G27" t="s">
         <v>18</v>
       </c>
       <c r="H27" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="I27" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="K27" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -2098,25 +2119,25 @@
         <v>72</v>
       </c>
       <c r="D28" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E28" t="s">
         <v>74</v>
       </c>
       <c r="F28" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G28" t="s">
         <v>18</v>
       </c>
       <c r="H28" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="I28" t="s">
         <v>87</v>
       </c>
       <c r="K28" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -2130,7 +2151,7 @@
         <v>82</v>
       </c>
       <c r="F29" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G29" t="s">
         <v>18</v>
@@ -2142,7 +2163,7 @@
         <v>91</v>
       </c>
       <c r="K29" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -2150,19 +2171,19 @@
         <v>85</v>
       </c>
       <c r="F30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G30" t="s">
         <v>18</v>
       </c>
       <c r="H30" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="I30" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K30" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -2173,19 +2194,19 @@
         <v>89</v>
       </c>
       <c r="F31" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G31" t="s">
         <v>18</v>
       </c>
       <c r="H31" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="I31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K31" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -2193,16 +2214,16 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D32" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F32" t="s">
         <v>17</v>
@@ -2211,33 +2232,33 @@
         <v>18</v>
       </c>
       <c r="H32" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I32" t="s">
-        <v>68</v>
+        <v>125</v>
       </c>
       <c r="J32" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K32" t="s">
         <v>21</v>
       </c>
       <c r="L32" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N32" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="C33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D33" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E33" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F33" t="s">
         <v>17</v>
@@ -2246,21 +2267,21 @@
         <v>18</v>
       </c>
       <c r="H33" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I33" t="s">
         <v>87</v>
       </c>
       <c r="K33" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="D34" t="s">
+        <v>142</v>
+      </c>
+      <c r="E34" t="s">
         <v>140</v>
-      </c>
-      <c r="E34" t="s">
-        <v>138</v>
       </c>
       <c r="F34" t="s">
         <v>17</v>
@@ -2269,13 +2290,13 @@
         <v>18</v>
       </c>
       <c r="H34" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I34" t="s">
         <v>32</v>
       </c>
       <c r="K34" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2283,16 +2304,16 @@
         <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C35" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D35" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E35" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F35" t="s">
         <v>17</v>
@@ -2301,13 +2322,13 @@
         <v>18</v>
       </c>
       <c r="H35" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="I35" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K35" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2315,16 +2336,16 @@
         <v>6</v>
       </c>
       <c r="B36" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D36" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F36" t="s">
         <v>17</v>
@@ -2333,13 +2354,13 @@
         <v>18</v>
       </c>
       <c r="H36" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="I36" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="K36" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2347,13 +2368,13 @@
         <v>7</v>
       </c>
       <c r="B37" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C37" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D37" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F37" t="s">
         <v>17</v>
@@ -2365,41 +2386,41 @@
         <v>47</v>
       </c>
       <c r="I37" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K37" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="D38" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F38" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G38" t="s">
         <v>18</v>
       </c>
       <c r="H38" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K38" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="C39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D39" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F39" t="s">
         <v>17</v>
@@ -2411,33 +2432,33 @@
         <v>47</v>
       </c>
       <c r="I39" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K39" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="D40" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E40" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F40" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G40" t="s">
         <v>18</v>
       </c>
       <c r="H40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K40" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2445,62 +2466,62 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C41" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D41" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E41" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G41" t="s">
         <v>18</v>
       </c>
       <c r="H41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I41" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="K41" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="D42" t="s">
+        <v>165</v>
+      </c>
+      <c r="E42" t="s">
+        <v>166</v>
+      </c>
+      <c r="F42" t="s">
+        <v>67</v>
+      </c>
+      <c r="G42" t="s">
+        <v>18</v>
+      </c>
+      <c r="H42" t="s">
         <v>163</v>
       </c>
-      <c r="E42" t="s">
+      <c r="I42" t="s">
         <v>164</v>
       </c>
-      <c r="F42" t="s">
-        <v>66</v>
-      </c>
-      <c r="G42" t="s">
-        <v>18</v>
-      </c>
-      <c r="H42" t="s">
-        <v>161</v>
-      </c>
-      <c r="I42" t="s">
-        <v>162</v>
-      </c>
       <c r="K42" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="C43" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D43" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F43" t="s">
         <v>17</v>
@@ -2509,21 +2530,21 @@
         <v>18</v>
       </c>
       <c r="H43" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I43" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="K43" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:11">
       <c r="D44" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E44" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F44" t="s">
         <v>38</v>
@@ -2532,13 +2553,13 @@
         <v>18</v>
       </c>
       <c r="H44" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I44" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="K44" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2557,25 +2578,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F1" t="s">
         <v>10</v>
       </c>
       <c r="G1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2586,19 +2607,19 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G2" t="s">
-        <v>180</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2606,22 +2627,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F3" t="s">
         <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -2629,22 +2650,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="G4" t="s">
-        <v>99</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -2652,19 +2673,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F5" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
         <v>33</v>
@@ -2682,40 +2703,40 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="I1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="J1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="K1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="L1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2723,37 +2744,37 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="K2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -2761,37 +2782,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D3" t="s">
+        <v>217</v>
+      </c>
+      <c r="E3" t="s">
+        <v>210</v>
+      </c>
+      <c r="F3" t="s">
+        <v>211</v>
+      </c>
+      <c r="G3" t="s">
+        <v>212</v>
+      </c>
+      <c r="H3" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" t="s">
+        <v>218</v>
+      </c>
+      <c r="K3" t="s">
         <v>215</v>
       </c>
-      <c r="E3" t="s">
-        <v>208</v>
-      </c>
-      <c r="F3" t="s">
-        <v>209</v>
-      </c>
-      <c r="G3" t="s">
-        <v>210</v>
-      </c>
-      <c r="H3" t="s">
-        <v>211</v>
-      </c>
-      <c r="I3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3" t="s">
-        <v>216</v>
-      </c>
-      <c r="K3" t="s">
-        <v>213</v>
-      </c>
       <c r="L3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -2799,37 +2820,37 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -2837,34 +2858,34 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D5" t="s">
+        <v>226</v>
+      </c>
+      <c r="E5" t="s">
+        <v>210</v>
+      </c>
+      <c r="F5" t="s">
+        <v>211</v>
+      </c>
+      <c r="G5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H5" t="s">
+        <v>222</v>
+      </c>
+      <c r="I5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K5" t="s">
         <v>224</v>
       </c>
-      <c r="E5" t="s">
-        <v>208</v>
-      </c>
-      <c r="F5" t="s">
-        <v>209</v>
-      </c>
-      <c r="G5" t="s">
-        <v>210</v>
-      </c>
-      <c r="H5" t="s">
-        <v>220</v>
-      </c>
-      <c r="I5" t="s">
-        <v>66</v>
-      </c>
-      <c r="K5" t="s">
-        <v>222</v>
-      </c>
       <c r="L5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -2872,37 +2893,37 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="K6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2910,37 +2931,37 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C7" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D7" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H7" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J7" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="K7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L7" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2948,37 +2969,37 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C8" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J8" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="K8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L8" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2986,34 +3007,34 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D9" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G9" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J9" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K9" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L9" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -3021,34 +3042,34 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D10" t="s">
+        <v>242</v>
+      </c>
+      <c r="E10" t="s">
+        <v>210</v>
+      </c>
+      <c r="F10" t="s">
+        <v>211</v>
+      </c>
+      <c r="G10" t="s">
+        <v>212</v>
+      </c>
+      <c r="H10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J10" t="s">
         <v>240</v>
       </c>
-      <c r="E10" t="s">
-        <v>208</v>
-      </c>
-      <c r="F10" t="s">
-        <v>209</v>
-      </c>
-      <c r="G10" t="s">
-        <v>210</v>
-      </c>
-      <c r="H10" t="s">
-        <v>220</v>
-      </c>
-      <c r="J10" t="s">
-        <v>238</v>
-      </c>
       <c r="K10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L10" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -3056,37 +3077,37 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C11" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I11" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J11" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="K11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -3094,37 +3115,37 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C12" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D12" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E12" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F12" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G12" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H12" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -3132,22 +3153,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C13" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D13" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H13" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="L13" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -3155,28 +3176,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C14" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E14" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F14" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H14" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J14" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -3184,28 +3205,28 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C15" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D15" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E15" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F15" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H15" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J15" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="L15" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -3213,28 +3234,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C16" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D16" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F16" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H16" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J16" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="L16" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -3242,28 +3263,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C17" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D17" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E17" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F17" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H17" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="I17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J17" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -3271,28 +3292,28 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C18" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D18" t="s">
+        <v>270</v>
+      </c>
+      <c r="E18" t="s">
+        <v>210</v>
+      </c>
+      <c r="F18" t="s">
+        <v>267</v>
+      </c>
+      <c r="H18" t="s">
         <v>268</v>
       </c>
-      <c r="E18" t="s">
-        <v>208</v>
-      </c>
-      <c r="F18" t="s">
-        <v>265</v>
-      </c>
-      <c r="H18" t="s">
-        <v>266</v>
-      </c>
       <c r="I18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J18" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -3300,28 +3321,28 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C19" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D19" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E19" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>